<commit_message>
added space in views
also made it so that example.xlsx is kept in sync with example.esm
</commit_message>
<xml_diff>
--- a/test/inputs/example.xlsx
+++ b/test/inputs/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E422B4F2-2C9A-AB4D-AD72-F1D17E1D69EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C437785-668A-DF4F-B0D7-8CA5B08AAF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19140" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19120" activeTab="4" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
   <sheets>
     <sheet name="Samples" sheetId="1" r:id="rId1"/>
@@ -120,9 +120,6 @@
     <t>mega</t>
   </si>
   <si>
-    <t>first_group,second_group</t>
-  </si>
-  <si>
     <t>plate_01_A[1:3]</t>
   </si>
   <si>
@@ -157,6 +154,9 @@
   </si>
   <si>
     <t>FSC_H,SSC_H,FL1_H,FL1_H,FL3_H,FL1_A,FL4_H</t>
+  </si>
+  <si>
+    <t>first_group, second_group</t>
   </si>
 </sst>
 </file>
@@ -574,10 +574,10 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -591,7 +591,7 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -616,10 +616,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
         <v>34</v>
-      </c>
-      <c r="B1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -646,7 +646,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -654,7 +654,7 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -662,7 +662,7 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -670,7 +670,7 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -700,7 +700,7 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -708,7 +708,7 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -726,7 +726,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -782,7 +782,7 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update calibrate to work with missing data
this also means we can remove colmean for ESM and replace with mean(eachcol(...))
</commit_message>
<xml_diff>
--- a/test/inputs/example.xlsx
+++ b/test/inputs/example.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C437785-668A-DF4F-B0D7-8CA5B08AAF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3074D74-49B1-6044-B5BB-DFD307C131AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19120" activeTab="4" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="18940" activeTab="3" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
   <sheets>
     <sheet name="Samples" sheetId="1" r:id="rId1"/>
@@ -129,12 +129,6 @@
     <t>plate_01_A[1,5,9]</t>
   </si>
   <si>
-    <t>hcat(first_group.flo,second_group.flo).-colmean(third_group.flo)</t>
-  </si>
-  <si>
-    <t>hcat(first_group.OD,second_group.OD).-colmean(third_group.OD)</t>
-  </si>
-  <si>
     <t>generic</t>
   </si>
   <si>
@@ -157,6 +151,12 @@
   </si>
   <si>
     <t>first_group, second_group</t>
+  </si>
+  <si>
+    <t>hcat(first_group.OD,second_group.OD).-mean(eachcol(third_group.OD))</t>
+  </si>
+  <si>
+    <t>hcat(first_group.flo,second_group.flo).-mean(eachcol(third_group.flo))</t>
   </si>
 </sst>
 </file>
@@ -574,10 +574,10 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -591,7 +591,7 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -616,10 +616,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -646,7 +646,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -700,7 +700,7 @@
         <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -708,7 +708,7 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -726,7 +726,7 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -782,7 +782,7 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>